<commit_message>
Optimize configuration for multi-agent setups
</commit_message>
<xml_diff>
--- a/config/Configuration-Multi-Target-Heterogeneus.xlsx
+++ b/config/Configuration-Multi-Target-Heterogeneus.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="272">
   <si>
     <t xml:space="preserve">GENERAL CONFIGURATION</t>
   </si>
@@ -76,129 +76,129 @@
     <t xml:space="preserve">ENVIRONMENT00</t>
   </si>
   <si>
+    <t xml:space="preserve">GROUP02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-150.0, 150.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(30.0, 150.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PX4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(13/12/2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(16:30:00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogeneus Configuration (B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heterogeneus Configuration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geopoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WindVel [m/s]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operational Conditions O1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(lat=35.9865559, lon=-5.8930106, alt=0.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Vx=3.0, Vy=1.5, Vz=0.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENVIRONMENT01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operational Conditions O2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Vx=4.0, Vy=3.5, Vz=0.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priority</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TrajectoryFolder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TARGET00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target Configuration L1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MetaHuman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TargetConfigurationL1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TARGET01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target Configuration L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TargetConfigurationL2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TARGET02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target Configuration L3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TargetConfigurationL3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TARGET03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target Configuration L4</t>
+  </si>
+  <si>
     <t xml:space="preserve">GROUP03</t>
   </si>
   <si>
-    <t xml:space="preserve">TEAM00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(-150.0, 150.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(30.0, 150.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PX4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(13/12/2024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(16:30:00)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogeneus Configuration (B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heterogeneus Configuration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geopoint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WindVel [m/s]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(lat=35.9865559, lon=-5.8930106, alt=0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Vx=3.0, Vy=1.5, Vz=0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENVIRONMENT01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Vx=4.0, Vy=3.5, Vz=0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TrajectoryFolder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MetaHuman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TargetConfigurationL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TargetConfigurationL2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TargetConfigurationL3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L4</t>
-  </si>
-  <si>
     <t xml:space="preserve">TargetConfigurationL4</t>
   </si>
   <si>
@@ -238,7 +238,7 @@
     <t xml:space="preserve">TRACKING00</t>
   </si>
   <si>
-    <t xml:space="preserve">DRONE02</t>
+    <t xml:space="preserve">DRONE00</t>
   </si>
   <si>
     <t xml:space="preserve">(X=10.0, Y=0.0, Z=0.0)</t>
@@ -256,25 +256,37 @@
     <t xml:space="preserve">Type A Agent Homogeneus 2</t>
   </si>
   <si>
+    <t xml:space="preserve">TRACKING01</t>
+  </si>
+  <si>
     <t xml:space="preserve">(X=-10.0, Y=0.0, Z=0.0)</t>
   </si>
   <si>
+    <t xml:space="preserve">tcp://127.0.0.1:5501</t>
+  </si>
+  <si>
     <t xml:space="preserve">AGENT02</t>
   </si>
   <si>
     <t xml:space="preserve">Type A Agent Homogeneus 3</t>
   </si>
   <si>
+    <t xml:space="preserve">TRACKING02</t>
+  </si>
+  <si>
     <t xml:space="preserve">(X=0.0, Y=10.0, Z=0.0)</t>
   </si>
   <si>
+    <t xml:space="preserve">tcp://127.0.0.1:5502</t>
+  </si>
+  <si>
     <t xml:space="preserve">AGENT03</t>
   </si>
   <si>
     <t xml:space="preserve">Type B Agent Homogeneus 1</t>
   </si>
   <si>
-    <t xml:space="preserve">TRACKING01</t>
+    <t xml:space="preserve">TRACKING03</t>
   </si>
   <si>
     <t xml:space="preserve">AGENT04</t>
@@ -283,19 +295,25 @@
     <t xml:space="preserve">Type B Agent Homogeneus 2</t>
   </si>
   <si>
+    <t xml:space="preserve">TRACKING04</t>
+  </si>
+  <si>
     <t xml:space="preserve">AGENT05</t>
   </si>
   <si>
     <t xml:space="preserve">Type B Agent Homogeneus 3</t>
   </si>
   <si>
+    <t xml:space="preserve">TRACKING05</t>
+  </si>
+  <si>
     <t xml:space="preserve">AGENT06</t>
   </si>
   <si>
     <t xml:space="preserve">Type A Agent Heterogeneus</t>
   </si>
   <si>
-    <t xml:space="preserve">TRACKING02</t>
+    <t xml:space="preserve">TRACKING06</t>
   </si>
   <si>
     <t xml:space="preserve">AGENT07</t>
@@ -304,7 +322,7 @@
     <t xml:space="preserve">Type B Agent Heterogeneus</t>
   </si>
   <si>
-    <t xml:space="preserve">TRACKING03</t>
+    <t xml:space="preserve">TRACKING07</t>
   </si>
   <si>
     <t xml:space="preserve">ObservationSetID</t>
@@ -319,30 +337,54 @@
     <t xml:space="preserve">RefTargetSize</t>
   </si>
   <si>
-    <t xml:space="preserve">Multi-Camera Tracking (2 Cameras)</t>
+    <t xml:space="preserve">Multi-Camera 1 Tracking (2 Cameras)</t>
   </si>
   <si>
     <t xml:space="preserve">SET00</t>
   </si>
   <si>
-    <t xml:space="preserve">Multi-Window Tracking (2 Windows)</t>
+    <t xml:space="preserve">Multi-Camera 2 Tracking (2 Cameras)</t>
   </si>
   <si>
     <t xml:space="preserve">SET01</t>
   </si>
   <si>
-    <t xml:space="preserve">Multi-Camera Tracking (3 Cameras)</t>
+    <t xml:space="preserve">Multi-Camera 3 Tracking (2 Cameras)</t>
   </si>
   <si>
     <t xml:space="preserve">SET02</t>
   </si>
   <si>
-    <t xml:space="preserve">Multi-Window Tracking (3 Windows)</t>
+    <t xml:space="preserve">Multi-Window 1 Tracking (2 Windows)</t>
   </si>
   <si>
     <t xml:space="preserve">SET03</t>
   </si>
   <si>
+    <t xml:space="preserve">Multi-Window 2 Tracking (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-Window 3 Tracking (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-Camera 1 Tracking (3 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-Window 2 Tracking (3 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET07</t>
+  </si>
+  <si>
     <t xml:space="preserve">CameraID</t>
   </si>
   <si>
@@ -379,19 +421,19 @@
     <t xml:space="preserve">MULTICAMERA00</t>
   </si>
   <si>
-    <t xml:space="preserve">Central Head Multi-Camera (2 Cameras)</t>
+    <t xml:space="preserve">Central Head 1 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
     <t xml:space="preserve">CAM00</t>
   </si>
   <si>
-    <t xml:space="preserve">GIM01</t>
+    <t xml:space="preserve">GIM00</t>
   </si>
   <si>
     <t xml:space="preserve">Central</t>
   </si>
   <si>
-    <t xml:space="preserve">(X=0.0, Y=0.0, Z=-0.15)</t>
+    <t xml:space="preserve">(X=0.0, Y=0.0, Z=-0.05)</t>
   </si>
   <si>
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=90.0)</t>
@@ -412,7 +454,7 @@
     <t xml:space="preserve">MULTICAMERA01</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Head 1 Multi-Camera (2 Cameras)</t>
+    <t xml:space="preserve">Tracking Head 1.1 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
     <t xml:space="preserve">CAM01</t>
@@ -421,7 +463,7 @@
     <t xml:space="preserve">Tracking</t>
   </si>
   <si>
-    <t xml:space="preserve">(X=0.3, Y=0.0, Z=-0.15)</t>
+    <t xml:space="preserve">(X=0.3, Y=0.0, Z=-0.05)</t>
   </si>
   <si>
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=0.0)</t>
@@ -436,10 +478,10 @@
     <t xml:space="preserve">MULTICAMERA02</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Head 2 Multi-Camera (2 Cameras)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(X=0.0, Y=0.3, Z=-0.15)</t>
+    <t xml:space="preserve">Tracking Head 1.2 Multi-Camera (2 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(X=0.0, Y=0.3, Z=-0.05)</t>
   </si>
   <si>
     <t xml:space="preserve">udp://127.0.0.1:5002</t>
@@ -451,52 +493,136 @@
     <t xml:space="preserve">MULTICAMERA03</t>
   </si>
   <si>
-    <t xml:space="preserve">Central Head Multi-Window (2 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAM04</t>
+    <t xml:space="preserve">Central Head 2 Multi-Camera (2 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:5003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:6003</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA04</t>
   </si>
   <si>
-    <t xml:space="preserve">Central Head Multi-Camera (3 Cameras)</t>
+    <t xml:space="preserve">Tracking Head 2.1 Multi-Camera (2 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:5004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:6004</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA05</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Head 1 Multi-Camera (3 Cameras)</t>
+    <t xml:space="preserve">Tracking Head 2.2 Multi-Camera (2 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:5005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:6005</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA06</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Head 2 Multi-Camera (3 Cameras)</t>
+    <t xml:space="preserve">Central Head 3 Multi-Camera (2 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:5006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:6006</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA07</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Head 3 Multi-Camera (3 Cameras)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(X=-0.3, Y=0.0, Z=-0.15)</t>
+    <t xml:space="preserve">Tracking Head 3.1 Multi-Camera (2 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:5007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:6007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTICAMERA08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Head 3.2 Multi-Camera (2 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:5008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">udp://127.0.0.1:6008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTICAMERA09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Head 1 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAM02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTICAMERA10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Head 2 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Udp://127.0.0.1:6003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTICAMERA11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Head 3 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Udp://127.0.0.1:6006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTICAMERA12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Head 1 Multi-Camera (3 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTICAMERA13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Head 1.1 Multi-Camera (3 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTICAMERA14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Head 1.2 Multi-Camera (3 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTICAMERA15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Head 1.3 Multi-Camera (3 Cameras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(X=-0.3, Y=0.0, Z=-0.05)</t>
   </si>
   <si>
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=180.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTICAMERA08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Central Head Multi-Window (3 Windows)</t>
+    <t xml:space="preserve">MULTICAMERA16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Head 2 Multi-Window (3 Windows)</t>
   </si>
   <si>
     <t xml:space="preserve">Resolution [pix]</t>
@@ -514,34 +640,58 @@
     <t xml:space="preserve">MULTIWINDOW00</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Window 1 Multi-Window (2 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(480x270)</t>
+    <t xml:space="preserve">Tracking Window 1.1 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(240x135)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW01</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Window 2 Multi-Window (2 Windows)</t>
+    <t xml:space="preserve">Tracking Window 1.2 Multi-Window (2 Windows)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW02</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Window 1 Multi-Window (3 Windows)</t>
+    <t xml:space="preserve">Tracking Window 2.1 Multi-Window (2 Windows)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW03</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Window 2 Multi-Window (3 Windows)</t>
+    <t xml:space="preserve">Tracking Window 2.2 Multi-Window (2 Windows)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW04</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking Window 3 Multi-Window (3 Windows)</t>
+    <t xml:space="preserve">Tracking Window 3.1 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 3.2 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 2.1 Multi-Window (3 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 2.2 Multi-Window (3 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 2.3 Multi-Window (3 Windows)</t>
   </si>
   <si>
     <t xml:space="preserve">HARDWARE CATALOGS</t>
@@ -592,25 +742,10 @@
     <t xml:space="preserve">LoadFactor [W/kg]</t>
   </si>
   <si>
-    <t xml:space="preserve">DRONE00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hexacopter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(WhiteNoiseSigma=2.7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(AngularWhiteNoiseSigma=0.3, VelocityWhiteNoiseSigma=0.24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(EphIni=25, EpvIni=25, EphFin=0.1, EpvFin=0.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(WhiteNoiseSigma=0.005, WhiteNoiseBias=0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRONE01</t>
+    <t xml:space="preserve">x500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quadcopter</t>
   </si>
   <si>
     <t xml:space="preserve">(WhiteNoiseSigma=8.0)</t>
@@ -625,12 +760,6 @@
     <t xml:space="preserve">(WhiteNoiseSigma=0.02, WhiteNoiseBias=0)</t>
   </si>
   <si>
-    <t xml:space="preserve">x500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quadcopter</t>
-  </si>
-  <si>
     <t xml:space="preserve">SensorSize [mm]</t>
   </si>
   <si>
@@ -652,66 +781,42 @@
     <t xml:space="preserve">ActivePower [W]</t>
   </si>
   <si>
-    <t xml:space="preserve">Operational Conditions O1 (low-resolution central camera)</t>
+    <t xml:space="preserve">Low-Resolution Central Camera</t>
   </si>
   <si>
     <t xml:space="preserve">RGB</t>
   </si>
   <si>
+    <t xml:space="preserve">(1280x720)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(13.2x7.425)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-0.03, 0.002, 0.0, 0.0005, -0.0004)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(RandContrib=0.001, RandSize=100, RandSpeed=50000)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-Resolution Tracking Camera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(960x540)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-Resolution Central Camera</t>
+  </si>
+  <si>
     <t xml:space="preserve">(1920x1080)</t>
   </si>
   <si>
-    <t xml:space="preserve">(13.2x7.425)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(-0.03, 0.002, 0.0, 0.0005, -0.0004)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(RandContrib=0.001, RandSize=100, RandSpeed=50000)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O1 (low-resolution tracking camera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1280x720)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAM02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O2 (low-resolution central camera)</t>
-  </si>
-  <si>
     <t xml:space="preserve">(-0.08, 0.008, 0.0001, 0.002, -0.0015)</t>
   </si>
   <si>
     <t xml:space="preserve">(RandContrib=0.003, RandSize=200, RandSpeed=70000)</t>
   </si>
   <si>
-    <t xml:space="preserve">CAM03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O2 (low-resolution tracking camera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O1 (ultra-high-resolution camera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(3840x2160)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAM05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O2 (ultra-high-resolution camera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAM06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(7.6x4.275)</t>
-  </si>
-  <si>
     <t xml:space="preserve">EnableRoll</t>
   </si>
   <si>
@@ -730,9 +835,6 @@
     <t xml:space="preserve">Yaw</t>
   </si>
   <si>
-    <t xml:space="preserve">GIM00</t>
-  </si>
-  <si>
     <t xml:space="preserve">Default Gimbal</t>
   </si>
   <si>
@@ -743,15 +845,6 @@
   </si>
   <si>
     <t xml:space="preserve">(Min=-320.0, Max=320.0, Speed=270)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Min=-30.0, Max=30.0, Speed=100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Min=-45.0, Max=90.0, Speed=100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Min=-135.0, Max=135.0, Speed=100)</t>
   </si>
 </sst>
 </file>
@@ -1184,8 +1277,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table210" displayName="Table210" ref="A2:J6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A2:J6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table210" displayName="Table210" ref="A2:J12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A2:J12"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Name"/>
@@ -1255,8 +1348,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table2913" displayName="Table2913" ref="A2:R3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A2:R3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table2913" displayName="Table2913" ref="A2:R2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A2:R2"/>
   <tableColumns count="18">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Name"/>
@@ -1825,7 +1918,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:XFD17"/>
+  <dimension ref="A1:XFD1048576"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="2" width="29.34"/>
@@ -1841,7 +1934,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>171</v>
+        <v>221</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1862,62 +1955,62 @@
         <v>2</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>227</v>
+        <v>262</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>228</v>
+        <v>263</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>229</v>
+        <v>264</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>230</v>
+        <v>265</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>231</v>
+        <v>266</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>232</v>
+        <v>267</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>204</v>
+        <v>247</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>205</v>
+        <v>248</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>206</v>
+        <v>249</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>233</v>
+        <v>132</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>234</v>
+        <v>268</v>
       </c>
       <c r="C3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>235</v>
+        <v>269</v>
       </c>
       <c r="E3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>236</v>
+        <v>270</v>
       </c>
       <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>237</v>
+        <v>271</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.4</v>
@@ -1929,44 +2022,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="C4" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>238</v>
-      </c>
-      <c r="E4" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F4" s="21" t="s">
-        <v>239</v>
-      </c>
-      <c r="G4" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H4" s="21" t="s">
-        <v>240</v>
-      </c>
-      <c r="I4" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="J4" s="21" t="n">
-        <v>5</v>
-      </c>
-      <c r="K4" s="21" t="n">
-        <v>15</v>
-      </c>
-    </row>
+    <row r="4" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1979,7 +2035,7 @@
     <row r="14" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
@@ -2366,7 +2422,7 @@
         <v>51</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>43</v>
@@ -2378,7 +2434,7 @@
         <v>44</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
@@ -2441,13 +2497,13 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="C6" s="9" t="s">
         <v>55</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>15</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>43</v>
@@ -2668,13 +2724,13 @@
         <v>16</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="E4" s="18" t="s">
         <v>69</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G4" s="18" t="s">
         <v>71</v>
@@ -2689,27 +2745,27 @@
         <v>12000</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>16</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="E5" s="18" t="s">
         <v>69</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G5" s="18" t="s">
         <v>71</v>
@@ -2724,21 +2780,21 @@
         <v>12000</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E6" s="18" t="s">
         <v>69</v>
@@ -2764,22 +2820,22 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C7" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="E7" s="18" t="s">
         <v>69</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G7" s="18" t="s">
         <v>71</v>
@@ -2794,27 +2850,27 @@
         <v>12000</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C8" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>69</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G8" s="18" t="s">
         <v>71</v>
@@ -2829,21 +2885,21 @@
         <v>12000</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>69</v>
@@ -2869,22 +2925,22 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E10" s="18" t="s">
         <v>69</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G10" s="18" t="s">
         <v>71</v>
@@ -2899,7 +2955,7 @@
         <v>12000</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2962,16 +3018,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="H2" s="12"/>
       <c r="I2" s="12"/>
@@ -2990,10 +3046,10 @@
         <v>68</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D3" s="18" t="n">
         <v>0.2</v>
@@ -3012,13 +3068,13 @@
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D4" s="18" t="n">
         <v>0.2</v>
@@ -3034,16 +3090,21 @@
       <c r="XEW4" s="2"/>
       <c r="XEX4" s="2"/>
       <c r="XEY4" s="3"/>
+      <c r="XEZ4" s="0"/>
+      <c r="XFA4" s="0"/>
+      <c r="XFB4" s="0"/>
+      <c r="XFC4" s="0"/>
+      <c r="XFD4" s="0"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>0.2</v>
@@ -3059,16 +3120,21 @@
       <c r="XEW5" s="2"/>
       <c r="XEX5" s="2"/>
       <c r="XEY5" s="3"/>
+      <c r="XEZ5" s="0"/>
+      <c r="XFA5" s="0"/>
+      <c r="XFB5" s="0"/>
+      <c r="XFC5" s="0"/>
+      <c r="XFD5" s="0"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D6" s="18" t="n">
         <v>0.2</v>
@@ -3085,20 +3151,116 @@
       <c r="XEX6" s="2"/>
       <c r="XEY6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="XEV7" s="2"/>
+      <c r="XEW7" s="2"/>
+      <c r="XEX7" s="2"/>
+      <c r="XEY7" s="3"/>
+    </row>
+    <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="XEV8" s="2"/>
+      <c r="XEW8" s="2"/>
+      <c r="XEX8" s="2"/>
+      <c r="XEY8" s="3"/>
+    </row>
+    <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G9" s="2"/>
+      <c r="XEV9" s="2"/>
+      <c r="XEW9" s="2"/>
+      <c r="XEX9" s="2"/>
+      <c r="XEY9" s="3"/>
+    </row>
+    <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="XEV10" s="2"/>
+      <c r="XEW10" s="2"/>
+      <c r="XEX10" s="2"/>
+      <c r="XEY10" s="3"/>
+    </row>
     <row r="11" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3173,16 +3335,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="G2" s="17" t="s">
         <v>60</v>
@@ -3191,28 +3353,28 @@
         <v>61</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="M2" s="17" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="N2" s="17" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="O2" s="17" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="P2" s="17" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="Q2" s="12"/>
       <c r="R2" s="12"/>
@@ -3221,28 +3383,28 @@
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I3" s="18" t="n">
         <v>3</v>
@@ -3254,16 +3416,16 @@
         <v>3</v>
       </c>
       <c r="L3" s="18" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="O3" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P3" s="18" t="n">
         <v>37260</v>
@@ -3271,28 +3433,28 @@
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="I4" s="18" t="n">
         <v>8</v>
@@ -3304,45 +3466,45 @@
         <v>10</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="O4" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P4" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
-    <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="B5" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="H5" s="18" t="s">
         <v>135</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>128</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="H5" s="18" t="s">
-        <v>121</v>
       </c>
       <c r="I5" s="18" t="n">
         <v>8</v>
@@ -3354,45 +3516,45 @@
         <v>10</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="M5" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="N5" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="N5" s="18" t="s">
-        <v>124</v>
-      </c>
       <c r="O5" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P5" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I6" s="18" t="n">
         <v>3</v>
@@ -3404,95 +3566,103 @@
         <v>3</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>122</v>
+        <v>155</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>123</v>
+        <v>156</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="O6" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P6" s="18" t="n">
         <v>37260</v>
       </c>
-    </row>
-    <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
+    </row>
+    <row r="7" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="E7" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F7" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="C7" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>117</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>119</v>
-      </c>
       <c r="G7" s="18" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="I7" s="18" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="K7" s="18" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>122</v>
+        <v>159</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>123</v>
+        <v>160</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="O7" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P7" s="18" t="n">
         <v>37260</v>
       </c>
-    </row>
-    <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="12"/>
+      <c r="T7" s="12"/>
+    </row>
+    <row r="8" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I8" s="18" t="n">
         <v>8</v>
@@ -3504,95 +3674,103 @@
         <v>10</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>132</v>
+        <v>163</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>133</v>
+        <v>164</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="O8" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P8" s="18" t="n">
         <v>37260</v>
       </c>
-    </row>
-    <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12"/>
+      <c r="T8" s="12"/>
+    </row>
+    <row r="9" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="K9" s="18" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L9" s="18" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="M9" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="N9" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="N9" s="18" t="s">
-        <v>124</v>
-      </c>
       <c r="O9" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P9" s="18" t="n">
         <v>37260</v>
       </c>
-    </row>
-    <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+    </row>
+    <row r="10" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="I10" s="18" t="n">
         <v>8</v>
@@ -3604,79 +3782,479 @@
         <v>10</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="M10" s="18" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="O10" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P10" s="18" t="n">
         <v>37260</v>
       </c>
-    </row>
-    <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+    </row>
+    <row r="11" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I11" s="18" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="K11" s="18" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L11" s="18" t="s">
-        <v>122</v>
+        <v>175</v>
       </c>
       <c r="M11" s="18" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="N11" s="18" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="O11" s="18" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="P11" s="18" t="n">
         <v>37260</v>
       </c>
-    </row>
-    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="12"/>
+    </row>
+    <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="M12" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="N12" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="O12" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="P12" s="18" t="n">
+        <v>37260</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="M13" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="N13" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="O13" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="P13" s="18" t="n">
+        <v>37260</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G14" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="H14" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I14" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="M14" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="N14" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="O14" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="P14" s="18" t="n">
+        <v>37260</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="H15" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L15" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="M15" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="N15" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="O15" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="P15" s="18" t="n">
+        <v>37260</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="M16" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="N16" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="O16" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="P16" s="18" t="n">
+        <v>37260</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="J17" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K17" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L17" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="M17" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="N17" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="O17" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="P17" s="18" t="n">
+        <v>37260</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>194</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="J18" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K18" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L18" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="M18" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="N18" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="O18" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="P18" s="18" t="n">
+        <v>37260</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>196</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J19" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K19" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L19" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="M19" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="N19" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="O19" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="P19" s="18" t="n">
+        <v>37260</v>
+      </c>
+    </row>
     <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3752,22 +4330,22 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>156</v>
+        <v>198</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>157</v>
+        <v>199</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>158</v>
+        <v>200</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>159</v>
+        <v>201</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="XEV2" s="3"/>
       <c r="XEW2" s="3"/>
@@ -3781,16 +4359,16 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>160</v>
+        <v>202</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>161</v>
+        <v>203</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>162</v>
+        <v>204</v>
       </c>
       <c r="E3" s="18" t="n">
         <v>0.167</v>
@@ -3802,21 +4380,21 @@
         <v>0.583</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>163</v>
+        <v>205</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>164</v>
+        <v>206</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>162</v>
+        <v>204</v>
       </c>
       <c r="E4" s="18" t="n">
         <v>0.167</v>
@@ -3828,21 +4406,21 @@
         <v>0.583</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>165</v>
+        <v>207</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>166</v>
+        <v>208</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>162</v>
+        <v>204</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>0.167</v>
@@ -3854,21 +4432,21 @@
         <v>0.583</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>133</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>167</v>
+        <v>209</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>162</v>
+        <v>204</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>0.167</v>
@@ -3880,21 +4458,21 @@
         <v>0.583</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>138</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>169</v>
+        <v>211</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>170</v>
+        <v>212</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>162</v>
+        <v>204</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>0.167</v>
@@ -3906,20 +4484,112 @@
         <v>0.583</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H8" s="12"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H9" s="12"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H10" s="12"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H11" s="12"/>
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="18" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="H10" s="18" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="F11" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="18" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="H12" s="12"/>
@@ -3927,10 +4597,18 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="H13" s="12"/>
     </row>
-    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H17" s="12"/>
+    </row>
     <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3973,7 +4651,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R1048576"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="26.66"/>
@@ -3993,7 +4671,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>171</v>
+        <v>221</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -4024,60 +4702,60 @@
         <v>36</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>172</v>
+        <v>222</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>173</v>
+        <v>223</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>174</v>
+        <v>224</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>175</v>
+        <v>225</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>176</v>
+        <v>226</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>177</v>
+        <v>227</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>178</v>
+        <v>228</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>179</v>
+        <v>229</v>
       </c>
       <c r="L2" s="20" t="s">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="M2" s="20" t="s">
-        <v>181</v>
+        <v>231</v>
       </c>
       <c r="N2" s="20" t="s">
-        <v>182</v>
+        <v>232</v>
       </c>
       <c r="O2" s="20" t="s">
-        <v>183</v>
+        <v>233</v>
       </c>
       <c r="P2" s="20" t="s">
-        <v>184</v>
+        <v>234</v>
       </c>
       <c r="Q2" s="20" t="s">
-        <v>185</v>
+        <v>235</v>
       </c>
       <c r="R2" s="20" t="s">
-        <v>186</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>187</v>
+        <v>69</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>30</v>
+        <v>237</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>188</v>
+        <v>238</v>
       </c>
       <c r="D3" s="21" t="n">
         <v>8</v>
@@ -4090,28 +4768,28 @@
         <v>1</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>189</v>
+        <v>239</v>
       </c>
       <c r="H3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="J3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K3" s="21" t="s">
-        <v>191</v>
+        <v>241</v>
       </c>
       <c r="L3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>192</v>
+        <v>242</v>
       </c>
       <c r="N3" s="21" t="n">
         <v>6.5</v>
@@ -4129,126 +4807,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
-        <v>193</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>188</v>
-      </c>
-      <c r="D4" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="F4" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="G4" s="21" t="s">
-        <v>194</v>
-      </c>
-      <c r="H4" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>195</v>
-      </c>
-      <c r="J4" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="K4" s="21" t="s">
-        <v>196</v>
-      </c>
-      <c r="L4" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="M4" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="N4" s="21" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="O4" s="21" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="P4" s="21" t="n">
-        <v>400</v>
-      </c>
-      <c r="Q4" s="21" t="n">
-        <v>350</v>
-      </c>
-      <c r="R4" s="21" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>198</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>199</v>
-      </c>
-      <c r="D5" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="F5" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="G5" s="21" t="s">
-        <v>194</v>
-      </c>
-      <c r="H5" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I5" s="21" t="s">
-        <v>195</v>
-      </c>
-      <c r="J5" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="K5" s="21" t="s">
-        <v>196</v>
-      </c>
-      <c r="L5" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="M5" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="N5" s="21" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="O5" s="21" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="P5" s="21" t="n">
-        <v>400</v>
-      </c>
-      <c r="Q5" s="21" t="n">
-        <v>350</v>
-      </c>
-      <c r="R5" s="21" t="n">
-        <v>25</v>
-      </c>
-    </row>
+    <row r="4" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4262,8 +4822,8 @@
     <row r="16" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="18" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
@@ -4286,7 +4846,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:XFD22"/>
+  <dimension ref="A1:XFD1048576"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
@@ -4304,7 +4864,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>171</v>
+        <v>221</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -4328,28 +4888,28 @@
         <v>36</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>156</v>
+        <v>198</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>200</v>
+        <v>243</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>201</v>
+        <v>244</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>202</v>
+        <v>245</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>203</v>
+        <v>246</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>204</v>
+        <v>247</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>205</v>
+        <v>248</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>206</v>
+        <v>249</v>
       </c>
       <c r="XFB2" s="3"/>
       <c r="XFC2" s="3"/>
@@ -4357,29 +4917,29 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>207</v>
+        <v>250</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>208</v>
+        <v>251</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>209</v>
+        <v>252</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>210</v>
+        <v>253</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>211</v>
+        <v>254</v>
       </c>
       <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>212</v>
+        <v>255</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.5</v>
@@ -4393,29 +4953,29 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>213</v>
+        <v>256</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>208</v>
+        <v>251</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>214</v>
+        <v>257</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>210</v>
+        <v>253</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>211</v>
+        <v>254</v>
       </c>
       <c r="G4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>212</v>
+        <v>255</v>
       </c>
       <c r="I4" s="21" t="n">
         <v>0.5</v>
@@ -4429,29 +4989,29 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>216</v>
+        <v>258</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>208</v>
+        <v>251</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>209</v>
+        <v>259</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>210</v>
+        <v>253</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>217</v>
+        <v>260</v>
       </c>
       <c r="G5" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>218</v>
+        <v>261</v>
       </c>
       <c r="I5" s="21" t="n">
         <v>0.5</v>
@@ -4463,150 +5023,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
-        <v>219</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>214</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>210</v>
-      </c>
-      <c r="F6" s="21" t="s">
-        <v>217</v>
-      </c>
-      <c r="G6" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>218</v>
-      </c>
-      <c r="I6" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J6" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" s="21" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>141</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>221</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>222</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>210</v>
-      </c>
-      <c r="F7" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="G7" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H7" s="21" t="s">
-        <v>212</v>
-      </c>
-      <c r="I7" s="21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="J7" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="21" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>224</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>222</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>210</v>
-      </c>
-      <c r="F8" s="21" t="s">
-        <v>217</v>
-      </c>
-      <c r="G8" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H8" s="21" t="s">
-        <v>218</v>
-      </c>
-      <c r="I8" s="21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="J8" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="K8" s="21" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>225</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>209</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>226</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="G9" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H9" s="21" t="s">
-        <v>212</v>
-      </c>
-      <c r="I9" s="21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="J9" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" s="21" t="n">
-        <v>6</v>
-      </c>
-    </row>
+    <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="11" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4616,10 +5036,10 @@
     <row r="16" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="18" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>

</xml_diff>